<commit_message>
Allow dates to be specified as days
</commit_message>
<xml_diff>
--- a/pymsprog/data/MSprog_toydata.xlsx
+++ b/pymsprog/data/MSprog_toydata.xlsx
@@ -1,32 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11008"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unigeit-my.sharepoint.com/personal/noemi_montobbio_unige_it/Documents/DATA/MS-toydata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="8_{0735295F-EBB6-3147-8CD4-DBE8B2F66519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{417862CD-B414-5C45-87FA-B76977C6FD64}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_3E5C2CA66CFFDF860F1D1ACA98CD57E4922399BC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{025682E4-1382-894F-962A-43C332BD8FB8}"/>
   <bookViews>
-    <workbookView xWindow="2860" yWindow="1960" windowWidth="22260" windowHeight="13640" xr2:uid="{943C05E5-5E7A-BA4E-A364-564D85E80AF6}"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="visits" sheetId="1" r:id="rId1"/>
     <sheet name="relapses" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
     <t>id</t>
   </si>
@@ -39,14 +34,28 @@
   <si>
     <t>SDMT</t>
   </si>
+  <si>
+    <t>day</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,16 +84,16 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -96,14 +105,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -111,44 +116,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -176,31 +181,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -228,26 +216,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -256,616 +227,739 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0CCFB8-D016-0A4C-A58B-C7331717A1C7}">
-  <dimension ref="A1:D49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E49"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>44462</v>
       </c>
       <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
         <v>4.5</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>44503</v>
       </c>
       <c r="C3">
+        <v>41</v>
+      </c>
+      <c r="D3">
         <v>4.5</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>44580</v>
       </c>
       <c r="C4">
+        <v>118</v>
+      </c>
+      <c r="D4">
         <v>4.5</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>44678</v>
       </c>
       <c r="C5">
+        <v>216</v>
+      </c>
+      <c r="D5">
         <v>4.5</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>44754</v>
       </c>
       <c r="C6">
+        <v>292</v>
+      </c>
+      <c r="D6">
         <v>5.5</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>44871</v>
       </c>
       <c r="C7">
+        <v>409</v>
+      </c>
+      <c r="D7">
         <v>5.5</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>44905</v>
       </c>
       <c r="C8">
+        <v>443</v>
+      </c>
+      <c r="D8">
         <v>5.5</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="2">
         <v>44996</v>
       </c>
       <c r="C9">
+        <v>534</v>
+      </c>
+      <c r="D9">
         <v>5.5</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>44161</v>
       </c>
       <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
         <v>4</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>44195</v>
       </c>
       <c r="C11">
+        <v>34</v>
+      </c>
+      <c r="D11">
         <v>4</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>44279</v>
       </c>
       <c r="C12">
+        <v>118</v>
+      </c>
+      <c r="D12">
         <v>4.5</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="2">
         <v>44359</v>
       </c>
       <c r="C13">
+        <v>198</v>
+      </c>
+      <c r="D13">
         <v>5.5</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="2">
         <v>44443</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>282</v>
       </c>
       <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="2">
         <v>44532</v>
       </c>
       <c r="C15">
+        <v>371</v>
+      </c>
+      <c r="D15">
         <v>4.5</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="2">
         <v>44615</v>
       </c>
       <c r="C16">
+        <v>454</v>
+      </c>
+      <c r="D16">
         <v>4.5</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="2">
         <v>44700</v>
       </c>
       <c r="C17">
+        <v>539</v>
+      </c>
+      <c r="D17">
         <v>6</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <v>44801</v>
       </c>
       <c r="C18">
+        <v>640</v>
+      </c>
+      <c r="D18">
         <v>6</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="2">
         <v>44891</v>
       </c>
       <c r="C19">
+        <v>730</v>
+      </c>
+      <c r="D19">
         <v>6</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="2">
         <v>44487</v>
       </c>
       <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
         <v>3.5</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>3</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="2">
         <v>44531</v>
       </c>
       <c r="C21">
+        <v>44</v>
+      </c>
+      <c r="D21">
         <v>4.5</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>3</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="2">
         <v>44607</v>
       </c>
       <c r="C22">
+        <v>120</v>
+      </c>
+      <c r="D22">
         <v>3.5</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>3</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="2">
         <v>44807</v>
       </c>
       <c r="C23">
+        <v>320</v>
+      </c>
+      <c r="D23">
         <v>3.5</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>3</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="2">
         <v>44839</v>
       </c>
       <c r="C24">
+        <v>352</v>
+      </c>
+      <c r="D24">
         <v>3.5</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>3</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="2">
         <v>44917</v>
       </c>
       <c r="C25">
+        <v>430</v>
+      </c>
+      <c r="D25">
         <v>3</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>3</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="2">
         <v>44978</v>
       </c>
       <c r="C26">
+        <v>491</v>
+      </c>
+      <c r="D26">
         <v>3</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="2">
         <v>44457</v>
       </c>
       <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
         <v>4.5</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="2">
         <v>44534</v>
       </c>
       <c r="C28">
+        <v>77</v>
+      </c>
+      <c r="D28">
         <v>3.5</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="2">
         <v>44632</v>
       </c>
       <c r="C29">
+        <v>175</v>
+      </c>
+      <c r="D29">
         <v>3.5</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="2">
         <v>44761</v>
       </c>
       <c r="C30">
-        <v>5</v>
+        <v>304</v>
       </c>
       <c r="D30">
+        <v>5</v>
+      </c>
+      <c r="E30">
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="2">
         <v>44839</v>
       </c>
       <c r="C31">
-        <v>5</v>
+        <v>382</v>
       </c>
       <c r="D31">
+        <v>5</v>
+      </c>
+      <c r="E31">
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="2">
         <v>44942</v>
       </c>
       <c r="C32">
+        <v>485</v>
+      </c>
+      <c r="D32">
         <v>5.5</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>52</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="2">
         <v>45043</v>
       </c>
       <c r="C33">
-        <v>5</v>
+        <v>586</v>
       </c>
       <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>5</v>
       </c>
@@ -873,219 +967,267 @@
         <v>44361</v>
       </c>
       <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
         <v>4</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>5</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="2">
         <v>44451</v>
       </c>
       <c r="C35">
+        <v>90</v>
+      </c>
+      <c r="D35">
         <v>4</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>5</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="2">
         <v>44501</v>
       </c>
       <c r="C36">
-        <v>5</v>
+        <v>140</v>
       </c>
       <c r="D36">
+        <v>5</v>
+      </c>
+      <c r="E36">
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>5</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="2">
         <v>44578</v>
       </c>
       <c r="C37">
+        <v>217</v>
+      </c>
+      <c r="D37">
         <v>5.5</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>5</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="2">
         <v>44681</v>
       </c>
       <c r="C38">
-        <v>5</v>
+        <v>320</v>
       </c>
       <c r="D38">
+        <v>5</v>
+      </c>
+      <c r="E38">
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>5</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="2">
         <v>44748</v>
       </c>
       <c r="C39">
+        <v>387</v>
+      </c>
+      <c r="D39">
         <v>5.5</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>5</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="2">
         <v>44874</v>
       </c>
       <c r="C40">
+        <v>513</v>
+      </c>
+      <c r="D40">
         <v>5.5</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>54</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>5</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="2">
         <v>44910</v>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>549</v>
       </c>
       <c r="D41">
+        <v>5</v>
+      </c>
+      <c r="E41">
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>5</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>44998</v>
       </c>
       <c r="C42">
+        <v>637</v>
+      </c>
+      <c r="D42">
         <v>5.5</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>6</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>44487</v>
       </c>
       <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
         <v>5.5</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>6</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>44531</v>
       </c>
       <c r="C44">
+        <v>44</v>
+      </c>
+      <c r="D44">
         <v>5.5</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>64</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>6</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>44607</v>
       </c>
       <c r="C45">
+        <v>120</v>
+      </c>
+      <c r="D45">
         <v>4.5</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>64</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>6</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>44807</v>
       </c>
       <c r="C46">
+        <v>320</v>
+      </c>
+      <c r="D46">
         <v>4.5</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>63</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>6</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="2">
         <v>44839</v>
       </c>
       <c r="C47">
-        <v>5</v>
+        <v>352</v>
       </c>
       <c r="D47">
+        <v>5</v>
+      </c>
+      <c r="E47">
         <v>60</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>6</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="2">
         <v>44917</v>
       </c>
       <c r="C48">
+        <v>430</v>
+      </c>
+      <c r="D48">
         <v>6</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>6</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="2">
         <v>44978</v>
       </c>
       <c r="C49">
+        <v>491</v>
+      </c>
+      <c r="D49">
         <v>6</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>61</v>
       </c>
     </row>
@@ -1095,48 +1237,66 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34402647-452C-0345-86DC-C118F6D6A291}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="20.6640625" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>44359</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>44859</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>44896</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>6</v>
       </c>
       <c r="B5" s="2">
         <v>44913</v>
+      </c>
+      <c r="C5">
+        <v>426</v>
       </c>
     </row>
   </sheetData>

</xml_diff>